<commit_message>
Mise à jour tests fonctionnels : Keycloak SSO, schema PG, landing Pennylane
- Auth : mis à jour pour Keycloak SSO (plus email/password custom)
- +5 tests Keycloak SSO (OTP, SSO cross-app, refresh, JWKS)
- +5 tests Isolation Données (schema PG, conversations, historique)
- +5 tests Landing Page (Pennylane, responsive, footer, liens légaux)
- +3 tests Dashboard (stats bar, actions rapides, thème)
- Version 3.0 (119 → 137 tests)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CGI242_Tests_Fonctionnels.xlsx
+++ b/CGI242_Tests_Fonctionnels.xlsx
@@ -144,7 +144,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -166,11 +166,55 @@
         <color rgb="00E5E7EB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E5E7EB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E5E7EB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E5E7EB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E5E7EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E5E7EB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E5E7EB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E5E7EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -224,6 +268,8 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -590,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -610,29 +656,29 @@
           <t>NORMX Tax 2026 — Plan de Tests Fonctionnels</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="21" t="n"/>
+      <c r="H1" s="21" t="n"/>
+      <c r="I1" s="22" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>NORMX AI SAS  ·  Testeur : Christelle  ·  Version 2.0 (CGI + Code Social)  ·  119 tests</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
+          <t>NORMX AI SAS  ·  Testeur : Christelle  ·  Version 3.0 (Keycloak SSO + Schema PG + Landing Pennylane)</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="n"/>
+      <c r="C2" s="21" t="n"/>
+      <c r="D2" s="21" t="n"/>
+      <c r="E2" s="21" t="n"/>
+      <c r="F2" s="21" t="n"/>
+      <c r="G2" s="21" t="n"/>
+      <c r="H2" s="21" t="n"/>
+      <c r="I2" s="22" t="n"/>
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4">
@@ -1321,7 +1367,7 @@
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>🔐  Sécurité 2FA</t>
+          <t>🔐  Keycloak OTP</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -1354,149 +1400,311 @@
       </c>
       <c r="I21" s="10" t="inlineStr">
         <is>
-          <t>Sécurité 2FA</t>
+          <t>Keycloak SSO</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>🔑  Keycloak SSO</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>🔑</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>5</v>
+      </c>
+      <c r="D22">
+        <f>COUNTIFS('🧪 Tests'!A:A,I22,'🧪 Tests'!G:G,"✅ PASS")</f>
+        <v/>
+      </c>
+      <c r="E22">
+        <f>COUNTIFS('🧪 Tests'!A:A,I22,'🧪 Tests'!G:G,"❌ FAIL")</f>
+        <v/>
+      </c>
+      <c r="F22">
+        <f>COUNTIFS('🧪 Tests'!A:A,I22,'🧪 Tests'!G:G,"⚠️ PARTIEL")</f>
+        <v/>
+      </c>
+      <c r="G22">
+        <f>COUNTIFS('🧪 Tests'!A:A,I22,'🧪 Tests'!G:G,"☐ À tester")</f>
+        <v/>
+      </c>
+      <c r="H22">
+        <f>IF(C22&gt;0,ROUND((D22+F22*0.5)/C22*100,1)&amp;"%","0%")</f>
+        <v/>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Keycloak SSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="8" customHeight="1">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>🗄️  Isolation Données</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>🗄️</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D23">
+        <f>COUNTIFS('🧪 Tests'!A:A,I23,'🧪 Tests'!G:G,"✅ PASS")</f>
+        <v/>
+      </c>
+      <c r="E23">
+        <f>COUNTIFS('🧪 Tests'!A:A,I23,'🧪 Tests'!G:G,"❌ FAIL")</f>
+        <v/>
+      </c>
+      <c r="F23">
+        <f>COUNTIFS('🧪 Tests'!A:A,I23,'🧪 Tests'!G:G,"⚠️ PARTIEL")</f>
+        <v/>
+      </c>
+      <c r="G23">
+        <f>COUNTIFS('🧪 Tests'!A:A,I23,'🧪 Tests'!G:G,"☐ À tester")</f>
+        <v/>
+      </c>
+      <c r="H23">
+        <f>IF(C23&gt;0,ROUND((D23+F23*0.5)/C23*100,1)&amp;"%","0%")</f>
+        <v/>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Isolation Données</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>🌐  Landing Page</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>🌐</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24">
+        <f>COUNTIFS('🧪 Tests'!A:A,I24,'🧪 Tests'!G:G,"✅ PASS")</f>
+        <v/>
+      </c>
+      <c r="E24">
+        <f>COUNTIFS('🧪 Tests'!A:A,I24,'🧪 Tests'!G:G,"❌ FAIL")</f>
+        <v/>
+      </c>
+      <c r="F24">
+        <f>COUNTIFS('🧪 Tests'!A:A,I24,'🧪 Tests'!G:G,"⚠️ PARTIEL")</f>
+        <v/>
+      </c>
+      <c r="G24">
+        <f>COUNTIFS('🧪 Tests'!A:A,I24,'🧪 Tests'!G:G,"☐ À tester")</f>
+        <v/>
+      </c>
+      <c r="H24">
+        <f>IF(C24&gt;0,ROUND((D24+F24*0.5)/C24*100,1)&amp;"%","0%")</f>
+        <v/>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Landing Page</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>📊  Dashboard</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>📊</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25">
+        <f>COUNTIFS('🧪 Tests'!A:A,I25,'🧪 Tests'!G:G,"✅ PASS")</f>
+        <v/>
+      </c>
+      <c r="E25">
+        <f>COUNTIFS('🧪 Tests'!A:A,I25,'🧪 Tests'!G:G,"❌ FAIL")</f>
+        <v/>
+      </c>
+      <c r="F25">
+        <f>COUNTIFS('🧪 Tests'!A:A,I25,'🧪 Tests'!G:G,"⚠️ PARTIEL")</f>
+        <v/>
+      </c>
+      <c r="G25">
+        <f>COUNTIFS('🧪 Tests'!A:A,I25,'🧪 Tests'!G:G,"☐ À tester")</f>
+        <v/>
+      </c>
+      <c r="H25">
+        <f>IF(C25&gt;0,ROUND((D25+F25*0.5)/C25*100,1)&amp;"%","0%")</f>
+        <v/>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>📊  TOTAL GÉNÉRAL</t>
         </is>
       </c>
-      <c r="B22" s="14" t="n"/>
-      <c r="C22" s="14" t="n">
-        <v>119</v>
-      </c>
-      <c r="D22" s="14">
+      <c r="B26" s="14" t="n"/>
+      <c r="C26" s="14">
+        <f>SUM(C5:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="14">
         <f>COUNTIF('🧪 Tests'!G:G,"✅ PASS")</f>
         <v/>
       </c>
-      <c r="E22" s="14">
+      <c r="E26" s="14">
         <f>COUNTIF('🧪 Tests'!G:G,"❌ FAIL")</f>
         <v/>
       </c>
-      <c r="F22" s="14">
+      <c r="F26" s="14">
         <f>COUNTIF('🧪 Tests'!G:G,"⚠️ PARTIEL")</f>
         <v/>
       </c>
-      <c r="G22" s="14">
+      <c r="G26" s="14">
         <f>COUNTIF('🧪 Tests'!G:G,"☐ À tester")</f>
         <v/>
       </c>
-      <c r="H22" s="14">
+      <c r="H26" s="14">
         <f>IF(C22&gt;0,ROUND((D22+F22*0.5)/C22*100,1)&amp;"%","0%")</f>
         <v/>
       </c>
-      <c r="I22" s="14" t="n"/>
-    </row>
-    <row r="23" ht="8" customHeight="1"/>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="I26" s="14" t="n"/>
+    </row>
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>LÉGENDE DES STATUTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="16" t="inlineStr">
-        <is>
-          <t>☐ À tester</t>
-        </is>
-      </c>
-      <c r="B25" s="17" t="inlineStr">
-        <is>
-          <t>Test non encore exécuté</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="16" t="inlineStr">
-        <is>
-          <t>✅ PASS</t>
-        </is>
-      </c>
-      <c r="B26" s="17" t="inlineStr">
-        <is>
-          <t>Test réussi — comportement conforme</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="16" t="inlineStr">
-        <is>
-          <t>❌ FAIL</t>
-        </is>
-      </c>
-      <c r="B27" s="17" t="inlineStr">
-        <is>
-          <t>Test échoué — bug à corriger</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ PARTIEL</t>
-        </is>
-      </c>
-      <c r="B28" s="17" t="inlineStr">
-        <is>
-          <t>Test partiellement réussi — à surveiller</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t>🚫 N/A</t>
+          <t>☐ À tester</t>
         </is>
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>Test non applicable dans ce contexte</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="8" customHeight="1"/>
+          <t>Test non encore exécuté</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>✅ PASS</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>Test réussi — comportement conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="8" customHeight="1">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>❌ FAIL</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>Test échoué — bug à corriger</t>
+        </is>
+      </c>
+    </row>
     <row r="32">
-      <c r="A32" s="15" t="inlineStr">
-        <is>
-          <t>✅  CRITÈRES MISE EN PRODUCTION</t>
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ PARTIEL</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>Test partiellement réussi — à surveiller</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
         <is>
+          <t>🚫 N/A</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>Test non applicable dans ce contexte</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
+        <is>
+          <t>✅  CRITÈRES MISE EN PRODUCTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
           <t>Minimum requis</t>
         </is>
       </c>
-      <c r="B33" s="17" t="inlineStr">
+      <c r="B37" s="17" t="inlineStr">
         <is>
           <t>100% des tests CRITIQUE en PASS ou N/A</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
         <is>
           <t>Recommandé</t>
         </is>
       </c>
-      <c r="B34" s="17" t="inlineStr">
+      <c r="B38" s="17" t="inlineStr">
         <is>
           <t>80% de tous les tests en PASS</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
         <is>
           <t>Aucun bug BLOQUANT</t>
         </is>
       </c>
-      <c r="B35" s="17" t="inlineStr">
+      <c r="B39" s="17" t="inlineStr">
         <is>
           <t>Tous les bugs BLOQUANT doivent être CORRIGÉ avant lancement</t>
         </is>
@@ -1523,7 +1731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K122"/>
+  <dimension ref="A1:K140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1545,33 +1753,33 @@
           <t>NORMX Tax 2026 — Grille de Tests Fonctionnels Interactive</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="21" t="n"/>
+      <c r="H1" s="21" t="n"/>
+      <c r="I1" s="21" t="n"/>
+      <c r="J1" s="21" t="n"/>
+      <c r="K1" s="22" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Modifiez la colonne STATUT avec la liste déroulante · Ajoutez vos commentaires et bugs dans les colonnes I et J</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
+          <t>Modifiez la colonne STATUT avec la liste déroulante · Version 3.0 (Keycloak SSO + Schema PG + Landing Pennylane)</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="n"/>
+      <c r="C2" s="21" t="n"/>
+      <c r="D2" s="21" t="n"/>
+      <c r="E2" s="21" t="n"/>
+      <c r="F2" s="21" t="n"/>
+      <c r="G2" s="21" t="n"/>
+      <c r="H2" s="21" t="n"/>
+      <c r="I2" s="21" t="n"/>
+      <c r="J2" s="21" t="n"/>
+      <c r="K2" s="22" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -1643,17 +1851,17 @@
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Inscription nouveau compte</t>
+          <t>Inscription via Keycloak SSO</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Taper email + mot de passe → Appuyer sur 'S'inscrire'</t>
+          <t>Accéder à tax.normx-ai.com → Cliquer 'Créer un compte' → Formulaire Keycloak</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>Compte créé, email de confirmation envoyé, redirection écran accueil</t>
+          <t>Compte créé sur auth.normx-ai.com, OTP email envoyé, redirection vers l'app</t>
         </is>
       </c>
       <c r="F4" s="18" t="inlineStr">
@@ -1684,17 +1892,17 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>Connexion avec compte existant</t>
+          <t>Connexion Keycloak SSO</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Entrer identifiants corrects → Connexion</t>
+          <t>Accéder à tax.normx-ai.com → 'Se connecter' → Identifiants Keycloak</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Accès tableau de bord, session ouverte, nom affiché en haut</t>
+          <t>Token JWT reçu, accès dashboard, nom affiché, token stocké en localStorage</t>
         </is>
       </c>
       <c r="F5" s="18" t="inlineStr">
@@ -1725,17 +1933,17 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Mot de passe incorrect (3 tentatives)</t>
+          <t>Brute force protection Keycloak</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Entrer un mot de passe erroné 3 fois de suite</t>
+          <t>Entrer un mot de passe erroné 5 fois de suite sur auth.normx-ai.com</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Message d'erreur clair, blocage temporaire après 3 échecs</t>
+          <t>Compte temporairement bloqué par Keycloak, message d'erreur clair</t>
         </is>
       </c>
       <c r="F6" s="19" t="inlineStr">
@@ -1766,17 +1974,17 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>Réinitialisation mot de passe</t>
+          <t>Réinitialisation mot de passe Keycloak</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Cliquer 'Mot de passe oublié' → saisir email → valider</t>
+          <t>Cliquer 'Mot de passe oublié' sur auth.normx-ai.com → saisir email</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Email de réinitialisation reçu dans les 2 minutes</t>
+          <t>Email de réinitialisation envoyé via Keycloak SMTP</t>
         </is>
       </c>
       <c r="F7" s="19" t="inlineStr">
@@ -1807,17 +2015,17 @@
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>Déconnexion</t>
+          <t>Déconnexion Keycloak</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Aller dans Profil → Déconnexion</t>
+          <t>Menu profil → Déconnexion</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>Session fermée, retour à l'écran de connexion</t>
+          <t>Session Keycloak fermée, tokens supprimés, retour landing page</t>
         </is>
       </c>
       <c r="F8" s="11" t="inlineStr">
@@ -1848,17 +2056,17 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Accès sans connexion (lien direct)</t>
+          <t>Accès protégé sans token</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Tenter d'accéder à un article sans être connecté</t>
+          <t>Accéder directement à une URL API sans token Bearer</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Redirection vers l'écran de connexion</t>
+          <t>401 Unauthorized, redirection vers login Keycloak</t>
         </is>
       </c>
       <c r="F9" s="19" t="inlineStr">
@@ -6508,6 +6716,672 @@
       <c r="I122" s="10" t="n"/>
       <c r="J122" s="10" t="n"/>
       <c r="K122" s="10" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Keycloak SSO</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>KC-01</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>OTP obligatoire au login</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Se connecter → Keycloak demande le code OTP</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Code OTP par email requis, login impossible sans</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>CRITIQUE</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Keycloak SSO</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>KC-02</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>SSO entre Tax et Legal</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Se connecter sur tax.normx-ai.com → ouvrir legal.normx-ai.com</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Déjà connecté sur Legal sans re-login (même session Keycloak)</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Keycloak SSO</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>KC-03</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Refresh token automatique</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Rester connecté &gt; 5 min sans activité</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Token rafraîchi automatiquement, pas de déconnexion</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Keycloak SSO</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>KC-04</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Token expiré → refresh</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Attendre expiration du access token</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Refresh token utilisé pour obtenir un nouveau access token</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Keycloak SSO</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>KC-05</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Validation JWKS côté serveur</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Envoyer une requête API avec un token invalide</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>401 rejeté, validation via JWKS de auth.normx-ai.com</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>CRITIQUE</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Isolation Données</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>ISO-01</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Création schema par utilisateur</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Nouveau user se connecte pour la première fois</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Schema PostgreSQL créé automatiquement (user_&lt;keycloak_id&gt;)</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>CRITIQUE</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Isolation Données</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>ISO-02</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Isolation conversations entre users</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>User A crée une conversation IA → User B se connecte</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>User B ne voit pas les conversations de User A</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>CRITIQUE</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Isolation Données</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>ISO-03</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Isolation historique recherche</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>User A fait des recherches → User B se connecte</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>User B ne voit pas l'historique de recherche de User A</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Isolation Données</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>ISO-04</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Isolation alertes fiscales</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>User A a des alertes → User B se connecte</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>User B ne voit pas les alertes de User A</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Isolation Données</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>ISO-05</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Audit log par schema</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Effectuer des actions → vérifier audit_log</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Actions tracées dans le schema de l'utilisateur uniquement</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>NORMALE</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Landing Page</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>LAND-01</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Affichage landing Pennylane</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Accéder à tax.normx-ai.com sans être connecté</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Landing page style Pennylane avec hero, features, CTA</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Landing Page</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>LAND-02</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Bouton Connexion → Keycloak</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Cliquer 'Se connecter' sur la landing</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Redirection vers auth.normx-ai.com/realms/normx-ai</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>CRITIQUE</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Landing Page</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>LAND-03</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Responsive mobile landing</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Ouvrir tax.normx-ai.com sur mobile</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Landing adaptée mobile, pas de scroll horizontal</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Landing Page</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>LAND-04</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Footer bleu marine</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Scroller en bas de la landing</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Footer fond bleu marine (#1A3A5C), texte blanc</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>NORMALE</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Landing Page</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>LAND-05</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Liens CGU/mentions/confidentialité</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Cliquer les liens légaux dans le footer</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Pages légales accessibles (normx-ai.com ou in-app)</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>DASH-01</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Stats bar bleu marine/or</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Se connecter → observer la barre de stats</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Barre avec stats (articles, simulateurs, IA) en bleu marine/or</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>NORMALE</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>DASH-02</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Actions rapides 2x2</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Observer les actions rapides sur le dashboard</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>4 actions rapides en grille 2x2 en premier</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>NORMALE</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>DASH-03</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Thème cohérent or/bleu</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Naviguer dans l'application</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Couleurs uniformes : or (#D4A843), bleu marine (#1A3A5C)</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>NORMALE</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>☐ À tester</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:K3"/>
@@ -6551,14 +7425,14 @@
           <t>NORMX Tax 2026 — Registre des Bugs &amp; Besoins d'Évolution</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="21" t="n"/>
+      <c r="H1" s="21" t="n"/>
+      <c r="I1" s="22" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -6566,14 +7440,14 @@
           <t>Consignez ici tous les bugs détectés et besoins d'amélioration identifiés pendant les tests</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
+      <c r="B2" s="21" t="n"/>
+      <c r="C2" s="21" t="n"/>
+      <c r="D2" s="21" t="n"/>
+      <c r="E2" s="21" t="n"/>
+      <c r="F2" s="21" t="n"/>
+      <c r="G2" s="21" t="n"/>
+      <c r="H2" s="21" t="n"/>
+      <c r="I2" s="22" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -7364,8 +8238,8 @@
           <t>NORMX Tax 2026 — Guide d'utilisation du fichier de tests</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="22" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="16" t="inlineStr"/>
@@ -7378,8 +8252,6 @@
           <t>🎯  COMMENT UTILISER CE FICHIER</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr"/>
@@ -7496,8 +8368,6 @@
           <t>📊  TABLEAU DE BORD</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="16" t="inlineStr"/>
@@ -7549,8 +8419,6 @@
           <t>🔵  CODES PRIORITÉ</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="16" t="inlineStr"/>
@@ -7615,8 +8483,6 @@
           <t>✅  CRITÈRES MISE EN PRODUCTION</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr"/>

</xml_diff>